<commit_message>
acebet: pricing v3, $10K platform + tranches 0-500K $0.016 / 500K-1M $0.013 / 1M-2M $0.011 / 2M+ $0.010 = ~3 cents all-in at 680K; pricing slide redrawn, explainer sheet v2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
+++ b/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
@@ -625,12 +625,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0 to 240,000: $0.030 / 240,001 to 500,000: $0.025 / 500,001 to 1,000,000: $0.020 / above 1,000,000: $0.015</t>
+          <t>0 to 500,000: $0.016 / 500,001 to 1,000,000: $0.013 / 1,000,001 to 2,000,000: $0.011 / above 2,000,000: $0.010</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Top tranche sits at Spreedly's quoted ~1.5 cents: upside as they open Canada, Australia, France, Spain.</t>
+          <t>Target (German, 27-Oct): about 3 cents all-in at today's volume, platform fee included. Top tranche $0.010 = pricing policy floor (internal).</t>
         </is>
       </c>
     </row>
@@ -642,12 +642,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>See tab Calculator: $17,300 usage + $10,000 platform = $27,300 a month ($327,600 a year).</t>
+          <t>See tab Calculator: $10,340 usage + $10,000 platform = $20,340 a month ($244,080 a year).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Usage average $0.025 per transaction (the "2.5 cents" target). All-in with platform fee: $0.040.</t>
+          <t>All-in $0.0299 per transaction (the 3-cent target); $0.0152 before the platform fee.</t>
         </is>
       </c>
     </row>
@@ -693,12 +693,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Payouts (redemptions) and reconciliation across Breeze, Coinflow, Whop and Checkout.</t>
+          <t>Reconciliation across Breeze, Coinflow, Whop and Checkout, for further review.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Boris showed interest in reconciliation; payouts relevant because Whop payouts are buggy. Price later.</t>
+          <t>Boris showed interest in reconciliation; scope and price later. Payouts removed from the proposal.</t>
         </is>
       </c>
     </row>
@@ -710,12 +710,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Rates locked, tranches reviewed annually. Pricing valid 30 days, subject to final agreement.</t>
+          <t>36-month contract. Rates locked, tranches reviewed annually. Pricing valid 30 days, subject to final agreement.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Term length and minimums not stated yet.</t>
+          <t>Minimums and billing start date not stated yet.</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Our usage average ($0.025) sits between them; all-in ($0.040) equals PaymentIQ. Unknown whether their quotes include platform fees: ask.</t>
+          <t>Our all-in ($0.030) sits between them; usage only ($0.015) matches Spreedly. Unknown whether their quotes include platform fees: ask.</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Policy floor is $0.01 per transaction; top tranche $0.015 is above it.</t>
+          <t>Policy floor is $0.01 per transaction; tranche 4 sits on it and tranche 3 ($0.011) just above.</t>
         </is>
       </c>
     </row>
@@ -861,13 +861,13 @@
         <v>0</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>240000</v>
+        <v>500000</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.03</v>
+        <v>0.016</v>
       </c>
       <c r="E6" s="6">
-        <f>MAX(0,MIN($B$2,240000)-0)</f>
+        <f>MAX(0,MIN($B$2,500000)-0)</f>
         <v/>
       </c>
       <c r="F6" s="8">
@@ -882,16 +882,16 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>240001</v>
+        <v>500001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.025</v>
+        <v>0.013</v>
       </c>
       <c r="E7" s="6">
-        <f>MAX(0,MIN($B$2,500000)-240000)</f>
+        <f>MAX(0,MIN($B$2,1000000)-500000)</f>
         <v/>
       </c>
       <c r="F7" s="8">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>500001</v>
+        <v>1000001</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1000000</v>
+        <v>2000000</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.02</v>
+        <v>0.011</v>
       </c>
       <c r="E8" s="6">
-        <f>MAX(0,MIN($B$2,1000000)-500000)</f>
+        <f>MAX(0,MIN($B$2,2000000)-1000000)</f>
         <v/>
       </c>
       <c r="F8" s="8">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>1000001</v>
+        <v>2000001</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -938,10 +938,10 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="E9" s="6">
-        <f>MAX(0,$B$2-1000000)</f>
+        <f>MAX(0,$B$2-2000000)</f>
         <v/>
       </c>
       <c r="F9" s="8">
@@ -1108,7 +1108,7 @@
         <v>680000</v>
       </c>
       <c r="B2" s="8">
-        <f>MAX(0,MIN(A2,240000)-0)*0.03+MAX(0,MIN(A2,500000)-240000)*0.025+MAX(0,MIN(A2,1000000)-500000)*0.02+MAX(0,A2-1000000)*0.015</f>
+        <f>MAX(0,MIN(A2,500000)-0)*0.016+MAX(0,MIN(A2,1000000)-500000)*0.013+MAX(0,MIN(A2,2000000)-1000000)*0.011+MAX(0,A2-2000000)*0.01</f>
         <v/>
       </c>
       <c r="C2" s="8">
@@ -1133,7 +1133,7 @@
         <v>1000000</v>
       </c>
       <c r="B3" s="8">
-        <f>MAX(0,MIN(A3,240000)-0)*0.03+MAX(0,MIN(A3,500000)-240000)*0.025+MAX(0,MIN(A3,1000000)-500000)*0.02+MAX(0,A3-1000000)*0.015</f>
+        <f>MAX(0,MIN(A3,500000)-0)*0.016+MAX(0,MIN(A3,1000000)-500000)*0.013+MAX(0,MIN(A3,2000000)-1000000)*0.011+MAX(0,A3-2000000)*0.01</f>
         <v/>
       </c>
       <c r="C3" s="8">
@@ -1158,7 +1158,7 @@
         <v>1500000</v>
       </c>
       <c r="B4" s="8">
-        <f>MAX(0,MIN(A4,240000)-0)*0.03+MAX(0,MIN(A4,500000)-240000)*0.025+MAX(0,MIN(A4,1000000)-500000)*0.02+MAX(0,A4-1000000)*0.015</f>
+        <f>MAX(0,MIN(A4,500000)-0)*0.016+MAX(0,MIN(A4,1000000)-500000)*0.013+MAX(0,MIN(A4,2000000)-1000000)*0.011+MAX(0,A4-2000000)*0.01</f>
         <v/>
       </c>
       <c r="C4" s="8">
@@ -1183,7 +1183,7 @@
         <v>2000000</v>
       </c>
       <c r="B5" s="8">
-        <f>MAX(0,MIN(A5,240000)-0)*0.03+MAX(0,MIN(A5,500000)-240000)*0.025+MAX(0,MIN(A5,1000000)-500000)*0.02+MAX(0,A5-1000000)*0.015</f>
+        <f>MAX(0,MIN(A5,500000)-0)*0.016+MAX(0,MIN(A5,1000000)-500000)*0.013+MAX(0,MIN(A5,2000000)-1000000)*0.011+MAX(0,A5-2000000)*0.01</f>
         <v/>
       </c>
       <c r="C5" s="8">
@@ -1208,7 +1208,7 @@
         <v>3000000</v>
       </c>
       <c r="B6" s="8">
-        <f>MAX(0,MIN(A6,240000)-0)*0.03+MAX(0,MIN(A6,500000)-240000)*0.025+MAX(0,MIN(A6,1000000)-500000)*0.02+MAX(0,A6-1000000)*0.015</f>
+        <f>MAX(0,MIN(A6,500000)-0)*0.016+MAX(0,MIN(A6,1000000)-500000)*0.013+MAX(0,MIN(A6,2000000)-1000000)*0.011+MAX(0,A6-2000000)*0.01</f>
         <v/>
       </c>
       <c r="C6" s="8">

</xml_diff>

<commit_message>
acebet: pricing v5, $10K platform + 3 / 2.5 / 2 / 1.5 cents on 0-500K / 500K-1M / 1M-2M / 2M+ ($29,500/mo at 680K); pricing slide redrawn, explainer sheet v4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
+++ b/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
@@ -625,12 +625,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0 to 500,000: $0.016 / 500,001 to 1,000,000: $0.013 / 1,000,001 to 2,000,000: $0.011 / above 2,000,000: $0.010</t>
+          <t>0 to 500,000: $0.030 / 500,001 to 1,000,000: $0.025 / 1,000,001 to 2,000,000: $0.020 / above 2,000,000: $0.015</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Target (German, 27-Oct): about 3 cents all-in at today's volume, platform fee included. Top tranche $0.010 = pricing policy floor (internal).</t>
+          <t>Rates per German (27-Oct): 3, 2.5, 2 and 1.5 cents, platform fee on top. Top tranche sits at Spreedly's quoted ~1.5 cents.</t>
         </is>
       </c>
     </row>
@@ -642,12 +642,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>See tab Calculator: $10,340 usage + $10,000 platform = $20,340 a month ($244,080 a year).</t>
+          <t>See tab Calculator: $19,500 usage + $10,000 platform = $29,500 a month ($354,000 a year).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>All-in $0.0299 per transaction (the 3-cent target); $0.0152 before the platform fee.</t>
+          <t>Average $0.0287 per transaction before the platform fee; $0.0434 all-in.</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Our all-in ($0.030) sits between them; usage only ($0.015) matches Spreedly. Unknown whether their quotes include platform fees: ask.</t>
+          <t>Our usage average ($0.029) sits between them; all-in ($0.043) is about PaymentIQ. Unknown whether their quotes include platform fees: ask.</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Policy floor is $0.01 per transaction; tranche 4 sits on it and tranche 3 ($0.011) just above.</t>
+          <t>Policy floor is $0.01 per transaction; every tranche is above it (lowest $0.015).</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         <v>500000</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.016</v>
+        <v>0.03</v>
       </c>
       <c r="E6" s="6">
         <f>MAX(0,MIN($B$2,500000)-0)</f>
@@ -888,7 +888,7 @@
         <v>1000000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.013</v>
+        <v>0.025</v>
       </c>
       <c r="E7" s="6">
         <f>MAX(0,MIN($B$2,1000000)-500000)</f>
@@ -912,7 +912,7 @@
         <v>2000000</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.011</v>
+        <v>0.02</v>
       </c>
       <c r="E8" s="6">
         <f>MAX(0,MIN($B$2,2000000)-1000000)</f>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="E9" s="6">
         <f>MAX(0,$B$2-2000000)</f>
@@ -1108,7 +1108,7 @@
         <v>680000</v>
       </c>
       <c r="B2" s="8">
-        <f>MAX(0,MIN(A2,500000)-0)*0.016+MAX(0,MIN(A2,1000000)-500000)*0.013+MAX(0,MIN(A2,2000000)-1000000)*0.011+MAX(0,A2-2000000)*0.01</f>
+        <f>MAX(0,MIN(A2,500000)-0)*0.03+MAX(0,MIN(A2,1000000)-500000)*0.025+MAX(0,MIN(A2,2000000)-1000000)*0.02+MAX(0,A2-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C2" s="8">
@@ -1133,7 +1133,7 @@
         <v>1000000</v>
       </c>
       <c r="B3" s="8">
-        <f>MAX(0,MIN(A3,500000)-0)*0.016+MAX(0,MIN(A3,1000000)-500000)*0.013+MAX(0,MIN(A3,2000000)-1000000)*0.011+MAX(0,A3-2000000)*0.01</f>
+        <f>MAX(0,MIN(A3,500000)-0)*0.03+MAX(0,MIN(A3,1000000)-500000)*0.025+MAX(0,MIN(A3,2000000)-1000000)*0.02+MAX(0,A3-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C3" s="8">
@@ -1158,7 +1158,7 @@
         <v>1500000</v>
       </c>
       <c r="B4" s="8">
-        <f>MAX(0,MIN(A4,500000)-0)*0.016+MAX(0,MIN(A4,1000000)-500000)*0.013+MAX(0,MIN(A4,2000000)-1000000)*0.011+MAX(0,A4-2000000)*0.01</f>
+        <f>MAX(0,MIN(A4,500000)-0)*0.03+MAX(0,MIN(A4,1000000)-500000)*0.025+MAX(0,MIN(A4,2000000)-1000000)*0.02+MAX(0,A4-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C4" s="8">
@@ -1183,7 +1183,7 @@
         <v>2000000</v>
       </c>
       <c r="B5" s="8">
-        <f>MAX(0,MIN(A5,500000)-0)*0.016+MAX(0,MIN(A5,1000000)-500000)*0.013+MAX(0,MIN(A5,2000000)-1000000)*0.011+MAX(0,A5-2000000)*0.01</f>
+        <f>MAX(0,MIN(A5,500000)-0)*0.03+MAX(0,MIN(A5,1000000)-500000)*0.025+MAX(0,MIN(A5,2000000)-1000000)*0.02+MAX(0,A5-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C5" s="8">
@@ -1208,7 +1208,7 @@
         <v>3000000</v>
       </c>
       <c r="B6" s="8">
-        <f>MAX(0,MIN(A6,500000)-0)*0.016+MAX(0,MIN(A6,1000000)-500000)*0.013+MAX(0,MIN(A6,2000000)-1000000)*0.011+MAX(0,A6-2000000)*0.01</f>
+        <f>MAX(0,MIN(A6,500000)-0)*0.03+MAX(0,MIN(A6,1000000)-500000)*0.025+MAX(0,MIN(A6,2000000)-1000000)*0.02+MAX(0,A6-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C6" s="8">

</xml_diff>

<commit_message>
acebet: pricing v6, $10K platform + 2.5 / 2 / 1.5 cents on 0-1M / 1M-2M / 2M+ ($27,000/mo at 680K); pricing + included slides redrawn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
+++ b/Deals/Acebet/sheet/Acebet_proposal_explainer.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Platform fee $10,000/month flat + a rate per successful transaction in 4 tranches.</t>
+          <t>Platform fee $10,000/month flat + a rate per successful transaction in 3 tranches.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -625,12 +625,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0 to 500,000: $0.030 / 500,001 to 1,000,000: $0.025 / 1,000,001 to 2,000,000: $0.020 / above 2,000,000: $0.015</t>
+          <t>0 to 1,000,000: $0.025 / 1,000,001 to 2,000,000: $0.020 / above 2,000,000: $0.015</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Rates per German (27-Oct): 3, 2.5, 2 and 1.5 cents, platform fee on top. Top tranche sits at Spreedly's quoted ~1.5 cents.</t>
+          <t>Rates per German (27-Oct): 2.5, 2 and 1.5 cents, platform fee on top. Top tranche sits at Spreedly's quoted ~1.5 cents.</t>
         </is>
       </c>
     </row>
@@ -642,12 +642,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>See tab Calculator: $19,500 usage + $10,000 platform = $29,500 a month ($354,000 a year).</t>
+          <t>See tab Calculator: $17,000 usage + $10,000 platform = $27,000 a month ($324,000 a year).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Average $0.0287 per transaction before the platform fee; $0.0434 all-in.</t>
+          <t>Average $0.0250 per transaction before the platform fee; $0.0397 all-in.</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Our usage average ($0.029) sits between them; all-in ($0.043) is about PaymentIQ. Unknown whether their quotes include platform fees: ask.</t>
+          <t>Our usage average ($0.025) sits between them; all-in ($0.040) is about PaymentIQ. Unknown whether their quotes include platform fees: ask.</t>
         </is>
       </c>
     </row>
@@ -861,13 +861,13 @@
         <v>0</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.03</v>
+        <v>0.025</v>
       </c>
       <c r="E6" s="6">
-        <f>MAX(0,MIN($B$2,500000)-0)</f>
+        <f>MAX(0,MIN($B$2,1000000)-0)</f>
         <v/>
       </c>
       <c r="F6" s="8">
@@ -882,16 +882,16 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>500001</v>
+        <v>1000001</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1000000</v>
+        <v>2000000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
       <c r="E7" s="6">
-        <f>MAX(0,MIN($B$2,1000000)-500000)</f>
+        <f>MAX(0,MIN($B$2,2000000)-1000000)</f>
         <v/>
       </c>
       <c r="F7" s="8">
@@ -906,46 +906,22 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>1000001</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>2000000</v>
+        <v>2000001</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>no cap</t>
+        </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="E8" s="6">
-        <f>MAX(0,MIN($B$2,2000000)-1000000)</f>
+        <f>MAX(0,$B$2-2000000)</f>
         <v/>
       </c>
       <c r="F8" s="8">
         <f>E8*D8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Tranche 4</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>2000001</v>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>no cap</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="E9" s="6">
-        <f>MAX(0,$B$2-2000000)</f>
-        <v/>
-      </c>
-      <c r="F9" s="8">
-        <f>E9*D9</f>
         <v/>
       </c>
     </row>
@@ -959,11 +935,11 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="9">
-        <f>SUM(E6:E9)</f>
+        <f>SUM(E6:E8)</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUM(F6:F9)</f>
+        <f>SUM(F6:F8)</f>
         <v/>
       </c>
     </row>
@@ -1108,7 +1084,7 @@
         <v>680000</v>
       </c>
       <c r="B2" s="8">
-        <f>MAX(0,MIN(A2,500000)-0)*0.03+MAX(0,MIN(A2,1000000)-500000)*0.025+MAX(0,MIN(A2,2000000)-1000000)*0.02+MAX(0,A2-2000000)*0.015</f>
+        <f>MAX(0,MIN(A2,1000000)-0)*0.025+MAX(0,MIN(A2,2000000)-1000000)*0.02+MAX(0,A2-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C2" s="8">
@@ -1133,7 +1109,7 @@
         <v>1000000</v>
       </c>
       <c r="B3" s="8">
-        <f>MAX(0,MIN(A3,500000)-0)*0.03+MAX(0,MIN(A3,1000000)-500000)*0.025+MAX(0,MIN(A3,2000000)-1000000)*0.02+MAX(0,A3-2000000)*0.015</f>
+        <f>MAX(0,MIN(A3,1000000)-0)*0.025+MAX(0,MIN(A3,2000000)-1000000)*0.02+MAX(0,A3-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C3" s="8">
@@ -1158,7 +1134,7 @@
         <v>1500000</v>
       </c>
       <c r="B4" s="8">
-        <f>MAX(0,MIN(A4,500000)-0)*0.03+MAX(0,MIN(A4,1000000)-500000)*0.025+MAX(0,MIN(A4,2000000)-1000000)*0.02+MAX(0,A4-2000000)*0.015</f>
+        <f>MAX(0,MIN(A4,1000000)-0)*0.025+MAX(0,MIN(A4,2000000)-1000000)*0.02+MAX(0,A4-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C4" s="8">
@@ -1183,7 +1159,7 @@
         <v>2000000</v>
       </c>
       <c r="B5" s="8">
-        <f>MAX(0,MIN(A5,500000)-0)*0.03+MAX(0,MIN(A5,1000000)-500000)*0.025+MAX(0,MIN(A5,2000000)-1000000)*0.02+MAX(0,A5-2000000)*0.015</f>
+        <f>MAX(0,MIN(A5,1000000)-0)*0.025+MAX(0,MIN(A5,2000000)-1000000)*0.02+MAX(0,A5-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C5" s="8">
@@ -1208,7 +1184,7 @@
         <v>3000000</v>
       </c>
       <c r="B6" s="8">
-        <f>MAX(0,MIN(A6,500000)-0)*0.03+MAX(0,MIN(A6,1000000)-500000)*0.025+MAX(0,MIN(A6,2000000)-1000000)*0.02+MAX(0,A6-2000000)*0.015</f>
+        <f>MAX(0,MIN(A6,1000000)-0)*0.025+MAX(0,MIN(A6,2000000)-1000000)*0.02+MAX(0,A6-2000000)*0.015</f>
         <v/>
       </c>
       <c r="C6" s="8">

</xml_diff>